<commit_message>
Update: regenerate Task 4/5 tables after Green’s normalization fix
</commit_message>
<xml_diff>
--- a/task4-5/out/task5_comparison.xlsx
+++ b/task4-5/out/task5_comparison.xlsx
@@ -535,7 +535,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>corner</t>
+          <t>center</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -545,32 +545,32 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>0_none</t>
+          <t>U_uniform_total10C</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>100</t>
+          <t>100.7368318</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>0.198734</t>
+          <t>0.222891</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>100</t>
+          <t>100.7364815</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>-0.0003503</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>0.000</t>
+          <t>-0.002</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
@@ -580,14 +580,14 @@
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>8.785e-11</t>
+          <t>8.802e-11</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>face</t>
+          <t>center</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -597,32 +597,32 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>0_none</t>
+          <t>G_gradient_top1_bottom0</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>100</t>
+          <t>100.0368569</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>0.202418</t>
+          <t>0.222891</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>100</t>
+          <t>100.0368241</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>-3.28e-05</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>0.000</t>
+          <t>-0.000</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
@@ -632,7 +632,7 @@
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>8.785e-11</t>
+          <t>8.781e-11</t>
         </is>
       </c>
     </row>
@@ -649,12 +649,12 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>U_uniform_total10C</t>
+          <t>E_exp_center</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>102.947327</t>
+          <t>100.0127388</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -664,17 +664,17 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>100.7364815</t>
+          <t>100.0127179</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>-2.21085</t>
+          <t>-2.09e-05</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>-9.919</t>
+          <t>-0.000</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
@@ -684,71 +684,71 @@
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>8.802e-11</t>
+          <t>8.788e-11</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>corner</t>
+          <t>center</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>A_all+100</t>
+          <t>B_tb+100_lr-100</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>U_uniform_total10C</t>
+          <t>0_none</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>100.0370812</t>
+          <t>0.133</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>0.198734</t>
+          <t>0.222891</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>100.0092336</t>
+          <t>1.479046787e-14</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>-0.0278476</t>
+          <t>-0.133</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>-0.140</t>
+          <t>-0.597</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>253</t>
+          <t>257</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>8.802e-11</t>
+          <t>6.670e-11</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>face</t>
+          <t>center</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>A_all+100</t>
+          <t>B_tb+100_lr-100</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -758,37 +758,37 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>100.2630866</t>
+          <t>0.86983176</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>0.202418</t>
+          <t>0.222891</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>100.065536</t>
+          <t>0.7364814559</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>-0.197551</t>
+          <t>-0.13335</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>-0.976</t>
+          <t>-0.598</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>253</t>
+          <t>257</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>8.802e-11</t>
+          <t>6.676e-11</t>
         </is>
       </c>
     </row>
@@ -800,7 +800,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>A_all+100</t>
+          <t>B_tb+100_lr-100</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -810,7 +810,7 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>100.1474277</t>
+          <t>0.1698569198</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -820,131 +820,131 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>100.0368241</t>
+          <t>0.0368240728</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>-0.110604</t>
+          <t>-0.133033</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>-0.496</t>
+          <t>-0.597</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>253</t>
+          <t>257</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>8.781e-11</t>
+          <t>6.673e-11</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>corner</t>
+          <t>center</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>A_all+100</t>
+          <t>B_tb+100_lr-100</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>G_gradient_top1_bottom0</t>
+          <t>E_exp_center</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>100.0006155</t>
+          <t>0.1457387726</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>0.198734</t>
+          <t>0.222891</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>100.0001518</t>
+          <t>0.01271790454</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>-0.0004637</t>
+          <t>-0.133021</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>-0.002</t>
+          <t>-0.597</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>253</t>
+          <t>257</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>8.781e-11</t>
+          <t>6.672e-11</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>face</t>
+          <t>center</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>A_all+100</t>
+          <t>C_top+left+200_bottom0_right-400</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>G_gradient_top1_bottom0</t>
+          <t>0_none</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>100.0131432</t>
+          <t>-0.416</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>0.202418</t>
+          <t>0.546455</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>100.0032768</t>
+          <t>-9.713122103e-13</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>-0.0098664</t>
+          <t>0.416</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>-0.049</t>
+          <t>0.761</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>253</t>
+          <t>263</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>8.781e-11</t>
+          <t>7.133e-11</t>
         </is>
       </c>
     </row>
@@ -956,111 +956,111 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>A_all+100</t>
+          <t>C_top+left+200_bottom0_right-400</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>E_exp_center</t>
+          <t>U_uniform_total10C</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>100.0509551</t>
+          <t>0.32083176</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>0.222891</t>
+          <t>0.546455</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>100.0127179</t>
+          <t>0.7364814559</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>-0.0382372</t>
+          <t>0.41565</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>-0.172</t>
+          <t>0.761</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>253</t>
+          <t>263</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>8.788e-11</t>
+          <t>7.140e-11</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>corner</t>
+          <t>center</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>A_all+100</t>
+          <t>C_top+left+200_bottom0_right-400</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>E_exp_center</t>
+          <t>G_gradient_top1_bottom0</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>100.0001128</t>
+          <t>-0.3791430802</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>0.198734</t>
+          <t>0.546455</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>100.0000277</t>
+          <t>0.0368240728</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>-8.51e-05</t>
+          <t>0.415967</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>-0.000</t>
+          <t>0.761</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>253</t>
+          <t>263</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>8.788e-11</t>
+          <t>7.142e-11</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>face</t>
+          <t>center</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>A_all+100</t>
+          <t>C_top+left+200_bottom0_right-400</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -1070,49 +1070,49 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>100.0020303</t>
+          <t>-0.4032612274</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>0.202418</t>
+          <t>0.546455</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>100.0005033</t>
+          <t>0.01271790454</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>-0.001527</t>
+          <t>0.415979</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>-0.008</t>
+          <t>0.761</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>253</t>
+          <t>263</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>8.788e-11</t>
+          <t>7.134e-11</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>center</t>
+          <t>corner</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>B_tb+100_lr-100</t>
+          <t>A_all+100</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -1122,37 +1122,37 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>0.133</t>
+          <t>100</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>0.222891</t>
+          <t>0.198734</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>1.479046787e-14</t>
+          <t>100</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>-0.133</t>
+          <t>0</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>-0.597</t>
+          <t>0.000</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>257</t>
+          <t>253</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>6.670e-11</t>
+          <t>8.785e-11</t>
         </is>
       </c>
     </row>
@@ -1164,17 +1164,17 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>B_tb+100_lr-100</t>
+          <t>A_all+100</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>0_none</t>
+          <t>U_uniform_total10C</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>0.029</t>
+          <t>100.0092703</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
@@ -1184,131 +1184,131 @@
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>-1.726161819e-15</t>
+          <t>100.0092336</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>-0.029</t>
+          <t>-3.67e-05</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>-0.146</t>
+          <t>-0.000</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>257</t>
+          <t>253</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>6.670e-11</t>
+          <t>8.802e-11</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>face</t>
+          <t>corner</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>B_tb+100_lr-100</t>
+          <t>A_all+100</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>0_none</t>
+          <t>G_gradient_top1_bottom0</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>-93.366</t>
+          <t>100.0001539</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>0.202418</t>
+          <t>0.198734</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>-93.32424553</t>
+          <t>100.0001518</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>0.0417545</t>
+          <t>-2.1e-06</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>0.206</t>
+          <t>-0.000</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>257</t>
+          <t>253</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>6.670e-11</t>
+          <t>8.781e-11</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>center</t>
+          <t>corner</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>B_tb+100_lr-100</t>
+          <t>A_all+100</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>U_uniform_total10C</t>
+          <t>E_exp_center</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>3.08032704</t>
+          <t>100.0000282</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>0.222891</t>
+          <t>0.198734</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>0.7364814559</t>
+          <t>100.0000277</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>-2.34385</t>
+          <t>-5e-07</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>-10.516</t>
+          <t>-0.000</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>257</t>
+          <t>253</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>6.676e-11</t>
+          <t>8.788e-11</t>
         </is>
       </c>
     </row>
@@ -1325,12 +1325,12 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>U_uniform_total10C</t>
+          <t>0_none</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>0.06608116</t>
+          <t>0.029</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
@@ -1340,17 +1340,17 @@
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>0.009233554927</t>
+          <t>-1.726161819e-15</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>-0.0568476</t>
+          <t>-0.029</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>-0.286</t>
+          <t>-0.146</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
@@ -1360,14 +1360,14 @@
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>6.676e-11</t>
+          <t>6.670e-11</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>face</t>
+          <t>corner</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -1382,27 +1382,27 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>-93.10291344</t>
+          <t>0.03827029</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>0.202418</t>
+          <t>0.198734</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>-93.25870954</t>
+          <t>0.009233554927</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>-0.155796</t>
+          <t>-0.0290367</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>-0.770</t>
+          <t>-0.146</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
@@ -1419,7 +1419,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>center</t>
+          <t>corner</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -1434,27 +1434,27 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>0.2804276792</t>
+          <t>0.0291538721</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>0.222891</t>
+          <t>0.198734</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>0.0368240728</t>
+          <t>0.0001518409836</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>-0.243604</t>
+          <t>-0.029002</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>-1.093</t>
+          <t>-0.146</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
@@ -1481,12 +1481,12 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>G_gradient_top1_bottom0</t>
+          <t>E_exp_center</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>0.0296154884</t>
+          <t>0.0290282016</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
@@ -1496,17 +1496,17 @@
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>0.0001518409836</t>
+          <t>2.770389812e-05</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>-0.0294636</t>
+          <t>-0.0290005</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>-0.148</t>
+          <t>-0.146</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
@@ -1516,111 +1516,111 @@
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>6.673e-11</t>
+          <t>6.672e-11</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>face</t>
+          <t>corner</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>B_tb+100_lr-100</t>
+          <t>C_top+left+200_bottom0_right-400</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>G_gradient_top1_bottom0</t>
+          <t>0_none</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>-93.35285678</t>
+          <t>99.818</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>0.202418</t>
+          <t>0.281506</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>-93.32096873</t>
+          <t>99.82483712</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>0.031888</t>
+          <t>0.00683712</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>0.158</t>
+          <t>0.024</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>257</t>
+          <t>263</t>
         </is>
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>6.673e-11</t>
+          <t>7.133e-11</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>center</t>
+          <t>corner</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>B_tb+100_lr-100</t>
+          <t>C_top+left+200_bottom0_right-400</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>E_exp_center</t>
+          <t>U_uniform_total10C</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>0.1839550905</t>
+          <t>99.82727029</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>0.222891</t>
+          <t>0.281506</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>0.01271790454</t>
+          <t>99.83407067</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>-0.171237</t>
+          <t>0.00680038</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>-0.768</t>
+          <t>0.024</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>257</t>
+          <t>263</t>
         </is>
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>6.672e-11</t>
+          <t>7.140e-11</t>
         </is>
       </c>
     </row>
@@ -1632,59 +1632,59 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>B_tb+100_lr-100</t>
+          <t>C_top+left+200_bottom0_right-400</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>E_exp_center</t>
+          <t>G_gradient_top1_bottom0</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>0.02911280642</t>
+          <t>99.81815387</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>0.198734</t>
+          <t>0.281506</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>2.770389812e-05</t>
+          <t>99.82498896</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>-0.0290851</t>
+          <t>0.00683509</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>-0.146</t>
+          <t>0.024</t>
         </is>
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>257</t>
+          <t>263</t>
         </is>
       </c>
       <c r="J24" t="inlineStr">
         <is>
-          <t>6.672e-11</t>
+          <t>7.142e-11</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>face</t>
+          <t>corner</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>B_tb+100_lr-100</t>
+          <t>C_top+left+200_bottom0_right-400</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -1694,49 +1694,49 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>-93.3639697</t>
+          <t>99.8180282</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>0.202418</t>
+          <t>0.281506</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>-93.32374219</t>
+          <t>99.82486482</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>0.0402275</t>
+          <t>0.00683662</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>0.199</t>
+          <t>0.024</t>
         </is>
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>257</t>
+          <t>263</t>
         </is>
       </c>
       <c r="J25" t="inlineStr">
         <is>
-          <t>6.672e-11</t>
+          <t>7.134e-11</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>center</t>
+          <t>face</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>C_top+left+200_bottom0_right-400</t>
+          <t>A_all+100</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
@@ -1746,89 +1746,89 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>-0.416</t>
+          <t>100</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>0.546455</t>
+          <t>0.202418</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>-9.713122103e-13</t>
+          <t>100</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>0.416</t>
+          <t>0</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>0.761</t>
+          <t>0.000</t>
         </is>
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>263</t>
+          <t>253</t>
         </is>
       </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t>7.133e-11</t>
+          <t>8.785e-11</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>corner</t>
+          <t>face</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>C_top+left+200_bottom0_right-400</t>
+          <t>A_all+100</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>0_none</t>
+          <t>U_uniform_total10C</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>99.818</t>
+          <t>100.0657716</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>0.281506</t>
+          <t>0.202418</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>99.82483712</t>
+          <t>100.065536</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>0.00683712</t>
+          <t>-0.0002356</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>0.024</t>
+          <t>-0.001</t>
         </is>
       </c>
       <c r="I27" t="inlineStr">
         <is>
-          <t>263</t>
+          <t>253</t>
         </is>
       </c>
       <c r="J27" t="inlineStr">
         <is>
-          <t>7.133e-11</t>
+          <t>8.802e-11</t>
         </is>
       </c>
     </row>
@@ -1840,151 +1840,151 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>C_top+left+200_bottom0_right-400</t>
+          <t>A_all+100</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>0_none</t>
+          <t>G_gradient_top1_bottom0</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>192.594</t>
+          <t>100.0032858</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>0.405657</t>
+          <t>0.202418</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>192.5094638</t>
+          <t>100.0032768</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>-0.0845362</t>
+          <t>-9e-06</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>-0.208</t>
+          <t>-0.000</t>
         </is>
       </c>
       <c r="I28" t="inlineStr">
         <is>
-          <t>263</t>
+          <t>253</t>
         </is>
       </c>
       <c r="J28" t="inlineStr">
         <is>
-          <t>7.133e-11</t>
+          <t>8.781e-11</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>center</t>
+          <t>face</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>C_top+left+200_bottom0_right-400</t>
+          <t>A_all+100</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>U_uniform_total10C</t>
+          <t>E_exp_center</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>2.53132704</t>
+          <t>100.0005076</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>0.546455</t>
+          <t>0.202418</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>0.7364814559</t>
+          <t>100.0005033</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>-1.79485</t>
+          <t>-4.3e-06</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>-3.285</t>
+          <t>-0.000</t>
         </is>
       </c>
       <c r="I29" t="inlineStr">
         <is>
-          <t>263</t>
+          <t>253</t>
         </is>
       </c>
       <c r="J29" t="inlineStr">
         <is>
-          <t>7.140e-11</t>
+          <t>8.788e-11</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>corner</t>
+          <t>face</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>C_top+left+200_bottom0_right-400</t>
+          <t>B_tb+100_lr-100</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>U_uniform_total10C</t>
+          <t>0_none</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>99.85508116</t>
+          <t>-93.366</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>0.281506</t>
+          <t>0.202418</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>99.83407067</t>
+          <t>-93.32424553</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>-0.0210105</t>
+          <t>0.0417545</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>-0.075</t>
+          <t>0.206</t>
         </is>
       </c>
       <c r="I30" t="inlineStr">
         <is>
-          <t>263</t>
+          <t>257</t>
         </is>
       </c>
       <c r="J30" t="inlineStr">
         <is>
-          <t>7.140e-11</t>
+          <t>6.670e-11</t>
         </is>
       </c>
     </row>
@@ -1996,7 +1996,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>C_top+left+200_bottom0_right-400</t>
+          <t>B_tb+100_lr-100</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
@@ -2006,49 +2006,49 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>192.8570866</t>
+          <t>-93.30022836</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>0.405657</t>
+          <t>0.202418</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>192.5749998</t>
+          <t>-93.25870954</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>-0.282087</t>
+          <t>0.0415188</t>
         </is>
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>-0.695</t>
+          <t>0.205</t>
         </is>
       </c>
       <c r="I31" t="inlineStr">
         <is>
-          <t>263</t>
+          <t>257</t>
         </is>
       </c>
       <c r="J31" t="inlineStr">
         <is>
-          <t>7.140e-11</t>
+          <t>6.676e-11</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>center</t>
+          <t>face</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>C_top+left+200_bottom0_right-400</t>
+          <t>B_tb+100_lr-100</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
@@ -2058,89 +2058,89 @@
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>-0.2685723208</t>
+          <t>-93.3627142</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>0.546455</t>
+          <t>0.202418</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>0.0368240728</t>
+          <t>-93.32096873</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>0.305396</t>
+          <t>0.0417455</t>
         </is>
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>0.559</t>
+          <t>0.206</t>
         </is>
       </c>
       <c r="I32" t="inlineStr">
         <is>
-          <t>263</t>
+          <t>257</t>
         </is>
       </c>
       <c r="J32" t="inlineStr">
         <is>
-          <t>7.142e-11</t>
+          <t>6.673e-11</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>corner</t>
+          <t>face</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>C_top+left+200_bottom0_right-400</t>
+          <t>B_tb+100_lr-100</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>G_gradient_top1_bottom0</t>
+          <t>E_exp_center</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>99.81861549</t>
+          <t>-93.36549242</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>0.281506</t>
+          <t>0.202418</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>99.82498896</t>
+          <t>-93.32374219</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>0.00637347</t>
+          <t>0.0417502</t>
         </is>
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>0.023</t>
+          <t>0.206</t>
         </is>
       </c>
       <c r="I33" t="inlineStr">
         <is>
-          <t>263</t>
+          <t>257</t>
         </is>
       </c>
       <c r="J33" t="inlineStr">
         <is>
-          <t>7.142e-11</t>
+          <t>6.672e-11</t>
         </is>
       </c>
     </row>
@@ -2157,12 +2157,12 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>G_gradient_top1_bottom0</t>
+          <t>0_none</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>192.6071432</t>
+          <t>192.594</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
@@ -2172,17 +2172,17 @@
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>192.5127406</t>
+          <t>192.5094638</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>-0.0944026</t>
+          <t>-0.0845362</t>
         </is>
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>-0.233</t>
+          <t>-0.208</t>
         </is>
       </c>
       <c r="I34" t="inlineStr">
@@ -2192,14 +2192,14 @@
       </c>
       <c r="J34" t="inlineStr">
         <is>
-          <t>7.142e-11</t>
+          <t>7.133e-11</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>center</t>
+          <t>face</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -2209,32 +2209,32 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>E_exp_center</t>
+          <t>U_uniform_total10C</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>-0.3650449095</t>
+          <t>192.6597716</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>0.546455</t>
+          <t>0.405657</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>0.01271790454</t>
+          <t>192.5749998</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>0.377763</t>
+          <t>-0.0847718</t>
         </is>
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>0.691</t>
+          <t>-0.209</t>
         </is>
       </c>
       <c r="I35" t="inlineStr">
@@ -2244,14 +2244,14 @@
       </c>
       <c r="J35" t="inlineStr">
         <is>
-          <t>7.134e-11</t>
+          <t>7.140e-11</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>corner</t>
+          <t>face</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -2261,32 +2261,32 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>E_exp_center</t>
+          <t>G_gradient_top1_bottom0</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>99.81811281</t>
+          <t>192.5972858</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>0.281506</t>
+          <t>0.405657</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>99.82486482</t>
+          <t>192.5127406</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>0.00675201</t>
+          <t>-0.0845452</t>
         </is>
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>0.024</t>
+          <t>-0.208</t>
         </is>
       </c>
       <c r="I36" t="inlineStr">
@@ -2296,7 +2296,7 @@
       </c>
       <c r="J36" t="inlineStr">
         <is>
-          <t>7.134e-11</t>
+          <t>7.142e-11</t>
         </is>
       </c>
     </row>
@@ -2318,7 +2318,7 @@
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>192.5960303</t>
+          <t>192.5945076</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
@@ -2333,12 +2333,12 @@
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>-0.0860632</t>
+          <t>-0.0845405</t>
         </is>
       </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t>-0.212</t>
+          <t>-0.208</t>
         </is>
       </c>
       <c r="I37" t="inlineStr">

</xml_diff>